<commit_message>
- set misa default value - print source line on runtime error - update riscv-csr.xlsx
</commit_message>
<xml_diff>
--- a/riscv-csr.xlsx
+++ b/riscv-csr.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\archlinux\home\hd\riscv-simulator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\archlinux\home\hd\Desktop\work-github\riscv-simulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8B1451-E970-4672-9E00-9D3A033B451E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3797E01-FAC9-43DA-AD64-DEABBE4A1617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="464" activeTab="2" xr2:uid="{8293AE58-3985-422E-ACBE-0DE584F3F72C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="464" activeTab="3" xr2:uid="{8293AE58-3985-422E-ACBE-0DE584F3F72C}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR Table" sheetId="1" r:id="rId1"/>
     <sheet name="mstatus mstatush sstatus" sheetId="2" r:id="rId2"/>
     <sheet name="mip mie" sheetId="5" r:id="rId3"/>
-    <sheet name="mideleg medeleg medelegh" sheetId="6" r:id="rId4"/>
+    <sheet name="misa" sheetId="7" r:id="rId4"/>
+    <sheet name="mideleg medeleg medelegh" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="bin2hex_32">_xlfn.LAMBDA(_xlpm.bin_str,    _xlfn.LET(     _xlpm.padded, RIGHT(REPT("0", 32) &amp; _xlpm.bin_str, 32),     _xlfn.CONCAT(       BIN2HEX(MID(_xlpm.padded, 1, 8), 2),       BIN2HEX(MID(_xlpm.padded, 9, 8), 2),       BIN2HEX(MID(_xlpm.padded, 17, 8), 2),       BIN2HEX(MID(_xlpm.padded, 25, 8), 2)     )   ) )</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -87,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="246">
   <si>
     <t>misa</t>
   </si>
@@ -735,6 +736,96 @@
   </si>
   <si>
     <t>Delegateable</t>
+  </si>
+  <si>
+    <t>MXL</t>
+  </si>
+  <si>
+    <t>Writeable</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>01</t>
   </si>
 </sst>
 </file>
@@ -767,7 +858,7 @@
       <name val="Consolas"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -795,6 +886,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -863,7 +960,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -910,6 +1007,9 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -934,7 +1034,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1590,7 +1711,7 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -1618,7 +1739,7 @@
         <f>REPT(IF(I3="Yes",1,0),C3)</f>
         <v>000000000000000000000</v>
       </c>
-      <c r="L3" s="20" t="str" cm="1">
+      <c r="L3" s="21" t="str" cm="1">
         <f t="array" ref="L3">bin2hex_32(_xlfn.CONCAT(K3:K11))</f>
         <v>00000000</v>
       </c>
@@ -1628,7 +1749,7 @@
       <c r="N3" s="15"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="17"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="5">
         <v>10</v>
       </c>
@@ -1658,14 +1779,14 @@
         <f t="shared" ref="K4:K34" si="0">REPT(IF(I4="Yes",1,0),C4)</f>
         <v>0</v>
       </c>
-      <c r="L4" s="20"/>
+      <c r="L4" s="21"/>
       <c r="M4" s="5" t="s">
         <v>139</v>
       </c>
       <c r="N4" s="15"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="17"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="5">
         <v>9</v>
       </c>
@@ -1695,14 +1816,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L5" s="20"/>
+      <c r="L5" s="21"/>
       <c r="M5" s="5" t="s">
         <v>139</v>
       </c>
       <c r="N5" s="15"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="5">
         <v>8</v>
       </c>
@@ -1728,14 +1849,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L6" s="20"/>
+      <c r="L6" s="21"/>
       <c r="M6" s="5" t="s">
         <v>139</v>
       </c>
       <c r="N6" s="15"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="17"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="5">
         <v>7</v>
       </c>
@@ -1765,14 +1886,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L7" s="20"/>
+      <c r="L7" s="21"/>
       <c r="M7" s="5" t="s">
         <v>139</v>
       </c>
       <c r="N7" s="15"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="5">
         <v>6</v>
       </c>
@@ -1802,14 +1923,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L8" s="20"/>
+      <c r="L8" s="21"/>
       <c r="M8" s="5" t="s">
         <v>139</v>
       </c>
       <c r="N8" s="15"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="17"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="5">
         <v>5</v>
       </c>
@@ -1839,7 +1960,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L9" s="20"/>
+      <c r="L9" s="21"/>
       <c r="M9" s="5" t="s">
         <v>139</v>
       </c>
@@ -1847,7 +1968,7 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="5">
         <v>4</v>
       </c>
@@ -1877,14 +1998,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L10" s="20"/>
+      <c r="L10" s="21"/>
       <c r="M10" s="5" t="s">
         <v>139</v>
       </c>
       <c r="N10" s="15"/>
     </row>
     <row r="11" spans="1:15" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="18"/>
+      <c r="A11" s="19"/>
       <c r="B11" s="5" t="s">
         <v>53</v>
       </c>
@@ -1910,7 +2031,7 @@
         <f t="shared" si="0"/>
         <v>0000</v>
       </c>
-      <c r="L11" s="20"/>
+      <c r="L11" s="21"/>
       <c r="M11" s="5" t="s">
         <v>139</v>
       </c>
@@ -1918,7 +2039,7 @@
       <c r="O11" s="14"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="20" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="5">
@@ -1952,7 +2073,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L12" s="20" t="str" cm="1">
+      <c r="L12" s="21" t="str" cm="1">
         <f t="array" ref="L12">bin2hex_32(_xlfn.CONCAT(K12:K34))</f>
         <v>007E19AA</v>
       </c>
@@ -1960,13 +2081,13 @@
         <f>REPT(IF(AND(J12="Yes",I12="Yes"),1,0),C12)</f>
         <v>0</v>
       </c>
-      <c r="N12" s="21" t="str" cm="1">
+      <c r="N12" s="22" t="str" cm="1">
         <f t="array" ref="N12">bin2hex_32(_xlfn.CONCAT(M12:M34))</f>
         <v>000C0122</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
+      <c r="A13" s="20"/>
       <c r="B13" s="5" t="s">
         <v>46</v>
       </c>
@@ -1992,15 +2113,15 @@
         <f t="shared" si="0"/>
         <v>000000</v>
       </c>
-      <c r="L13" s="20"/>
+      <c r="L13" s="21"/>
       <c r="M13" s="1" t="str">
         <f t="shared" ref="M13:M34" si="1">REPT(IF(AND(J13="Yes",I13="Yes"),1,0),C13)</f>
         <v>000000</v>
       </c>
-      <c r="N13" s="22"/>
+      <c r="N13" s="23"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="5">
         <v>24</v>
       </c>
@@ -2032,15 +2153,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L14" s="20"/>
+      <c r="L14" s="21"/>
       <c r="M14" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N14" s="22"/>
+      <c r="N14" s="23"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
+      <c r="A15" s="20"/>
       <c r="B15" s="5">
         <v>23</v>
       </c>
@@ -2072,15 +2193,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L15" s="20"/>
+      <c r="L15" s="21"/>
       <c r="M15" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N15" s="22"/>
+      <c r="N15" s="23"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
+      <c r="A16" s="20"/>
       <c r="B16" s="5">
         <v>22</v>
       </c>
@@ -2112,15 +2233,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L16" s="20"/>
+      <c r="L16" s="21"/>
       <c r="M16" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N16" s="22"/>
+      <c r="N16" s="23"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
+      <c r="A17" s="20"/>
       <c r="B17" s="5">
         <v>21</v>
       </c>
@@ -2152,15 +2273,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L17" s="20"/>
+      <c r="L17" s="21"/>
       <c r="M17" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N17" s="22"/>
+      <c r="N17" s="23"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="5">
         <v>20</v>
       </c>
@@ -2192,15 +2313,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L18" s="20"/>
+      <c r="L18" s="21"/>
       <c r="M18" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N18" s="22"/>
+      <c r="N18" s="23"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
+      <c r="A19" s="20"/>
       <c r="B19" s="5">
         <v>19</v>
       </c>
@@ -2232,15 +2353,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L19" s="20"/>
+      <c r="L19" s="21"/>
       <c r="M19" s="1" t="str">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="N19" s="22"/>
+      <c r="N19" s="23"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="19"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="5">
         <v>18</v>
       </c>
@@ -2272,15 +2393,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L20" s="20"/>
+      <c r="L20" s="21"/>
       <c r="M20" s="1" t="str">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="N20" s="22"/>
+      <c r="N20" s="23"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="20"/>
       <c r="B21" s="5">
         <v>17</v>
       </c>
@@ -2312,15 +2433,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L21" s="20"/>
+      <c r="L21" s="21"/>
       <c r="M21" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N21" s="22"/>
+      <c r="N21" s="23"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="20"/>
       <c r="B22" s="5" t="s">
         <v>47</v>
       </c>
@@ -2352,15 +2473,15 @@
         <f t="shared" si="0"/>
         <v>00</v>
       </c>
-      <c r="L22" s="20"/>
+      <c r="L22" s="21"/>
       <c r="M22" s="1" t="str">
         <f t="shared" si="1"/>
         <v>00</v>
       </c>
-      <c r="N22" s="22"/>
+      <c r="N22" s="23"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="20"/>
       <c r="B23" s="5" t="s">
         <v>48</v>
       </c>
@@ -2392,15 +2513,15 @@
         <f t="shared" si="0"/>
         <v>00</v>
       </c>
-      <c r="L23" s="20"/>
+      <c r="L23" s="21"/>
       <c r="M23" s="1" t="str">
         <f t="shared" si="1"/>
         <v>00</v>
       </c>
-      <c r="N23" s="22"/>
+      <c r="N23" s="23"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="5" t="s">
         <v>49</v>
       </c>
@@ -2432,15 +2553,15 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="L24" s="20"/>
+      <c r="L24" s="21"/>
       <c r="M24" s="1" t="str">
         <f t="shared" si="1"/>
         <v>00</v>
       </c>
-      <c r="N24" s="22"/>
+      <c r="N24" s="23"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="20"/>
       <c r="B25" s="5" t="s">
         <v>138</v>
       </c>
@@ -2472,15 +2593,15 @@
         <f t="shared" si="0"/>
         <v>00</v>
       </c>
-      <c r="L25" s="20"/>
+      <c r="L25" s="21"/>
       <c r="M25" s="1" t="str">
         <f t="shared" si="1"/>
         <v>00</v>
       </c>
-      <c r="N25" s="22"/>
+      <c r="N25" s="23"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="20"/>
       <c r="B26" s="5">
         <v>8</v>
       </c>
@@ -2512,15 +2633,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L26" s="20"/>
+      <c r="L26" s="21"/>
       <c r="M26" s="1" t="str">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="N26" s="22"/>
+      <c r="N26" s="23"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="19"/>
+      <c r="A27" s="20"/>
       <c r="B27" s="5">
         <v>7</v>
       </c>
@@ -2552,15 +2673,15 @@
         <f>REPT(IF(I27="Yes",1,0),C27)</f>
         <v>1</v>
       </c>
-      <c r="L27" s="20"/>
+      <c r="L27" s="21"/>
       <c r="M27" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N27" s="22"/>
+      <c r="N27" s="23"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="19"/>
+      <c r="A28" s="20"/>
       <c r="B28" s="5">
         <v>6</v>
       </c>
@@ -2592,15 +2713,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L28" s="20"/>
+      <c r="L28" s="21"/>
       <c r="M28" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N28" s="22"/>
+      <c r="N28" s="23"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="19"/>
+      <c r="A29" s="20"/>
       <c r="B29" s="5">
         <v>5</v>
       </c>
@@ -2632,15 +2753,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L29" s="20"/>
+      <c r="L29" s="21"/>
       <c r="M29" s="1" t="str">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="N29" s="22"/>
+      <c r="N29" s="23"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="19"/>
+      <c r="A30" s="20"/>
       <c r="B30" s="5">
         <v>4</v>
       </c>
@@ -2666,15 +2787,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L30" s="20"/>
+      <c r="L30" s="21"/>
       <c r="M30" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N30" s="22"/>
+      <c r="N30" s="23"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="19"/>
+      <c r="A31" s="20"/>
       <c r="B31" s="5">
         <v>3</v>
       </c>
@@ -2706,15 +2827,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L31" s="20"/>
+      <c r="L31" s="21"/>
       <c r="M31" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N31" s="22"/>
+      <c r="N31" s="23"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="19"/>
+      <c r="A32" s="20"/>
       <c r="B32" s="5">
         <v>2</v>
       </c>
@@ -2740,15 +2861,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L32" s="20"/>
+      <c r="L32" s="21"/>
       <c r="M32" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N32" s="22"/>
+      <c r="N32" s="23"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="19"/>
+      <c r="A33" s="20"/>
       <c r="B33" s="5">
         <v>1</v>
       </c>
@@ -2780,15 +2901,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="L33" s="20"/>
+      <c r="L33" s="21"/>
       <c r="M33" s="1" t="str">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="N33" s="22"/>
+      <c r="N33" s="23"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="19"/>
+      <c r="A34" s="20"/>
       <c r="B34" s="5">
         <v>0</v>
       </c>
@@ -2814,12 +2935,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L34" s="20"/>
+      <c r="L34" s="21"/>
       <c r="M34" s="1" t="str">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N34" s="23"/>
+      <c r="N34" s="24"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
@@ -3165,6 +3286,510 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE4BF47-6E7D-46DC-BEF8-68A92150F968}">
+  <dimension ref="G3:K35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="6" width="9.140625" style="6"/>
+    <col min="7" max="7" width="6.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="6"/>
+    <col min="9" max="9" width="13.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="4" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G4" s="10">
+        <v>31</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="I4" s="30" t="s">
+        <v>245</v>
+      </c>
+      <c r="J4" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="32" t="str" cm="1">
+        <f t="array" ref="K4">bin2hex_32(_xlfn.CONCAT(I4:I35))</f>
+        <v>40141101</v>
+      </c>
+    </row>
+    <row r="5" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G5" s="10">
+        <v>30</v>
+      </c>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="32"/>
+    </row>
+    <row r="6" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G6" s="25">
+        <v>29</v>
+      </c>
+      <c r="H6" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" s="26" t="s">
+        <v>218</v>
+      </c>
+      <c r="J6" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="32"/>
+    </row>
+    <row r="7" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G7" s="25">
+        <v>28</v>
+      </c>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="32"/>
+    </row>
+    <row r="8" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G8" s="25">
+        <v>27</v>
+      </c>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="32"/>
+    </row>
+    <row r="9" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G9" s="25">
+        <v>26</v>
+      </c>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="32"/>
+    </row>
+    <row r="10" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G10" s="11">
+        <v>25</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="32"/>
+    </row>
+    <row r="11" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G11" s="11">
+        <v>24</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K11" s="32"/>
+    </row>
+    <row r="12" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G12" s="11">
+        <v>23</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" s="32"/>
+    </row>
+    <row r="13" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G13" s="11">
+        <v>22</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G14" s="11">
+        <v>21</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K14" s="32"/>
+    </row>
+    <row r="15" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G15" s="10">
+        <v>20</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="32"/>
+    </row>
+    <row r="16" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G16" s="11">
+        <v>19</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="32"/>
+    </row>
+    <row r="17" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G17" s="10">
+        <v>18</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" s="32"/>
+    </row>
+    <row r="18" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G18" s="11">
+        <v>17</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K18" s="32"/>
+    </row>
+    <row r="19" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G19" s="11">
+        <v>16</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J19" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K19" s="32"/>
+    </row>
+    <row r="20" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G20" s="11">
+        <v>15</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J20" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K20" s="32"/>
+    </row>
+    <row r="21" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G21" s="11">
+        <v>14</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K21" s="32"/>
+    </row>
+    <row r="22" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G22" s="11">
+        <v>13</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J22" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K22" s="32"/>
+    </row>
+    <row r="23" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G23" s="10">
+        <v>12</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="J23" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K23" s="32"/>
+    </row>
+    <row r="24" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G24" s="11">
+        <v>11</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J24" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K24" s="32"/>
+    </row>
+    <row r="25" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G25" s="11">
+        <v>10</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J25" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K25" s="32"/>
+    </row>
+    <row r="26" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G26" s="11">
+        <v>9</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="I26" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J26" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K26" s="32"/>
+    </row>
+    <row r="27" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G27" s="10">
+        <v>8</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="J27" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G28" s="11">
+        <v>7</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J28" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K28" s="32"/>
+    </row>
+    <row r="29" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G29" s="11">
+        <v>6</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J29" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K29" s="32"/>
+    </row>
+    <row r="30" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G30" s="11">
+        <v>5</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G31" s="11">
+        <v>4</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K31" s="32"/>
+    </row>
+    <row r="32" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G32" s="11">
+        <v>3</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J32" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K32" s="32"/>
+    </row>
+    <row r="33" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G33" s="11">
+        <v>2</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J33" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K33" s="32"/>
+    </row>
+    <row r="34" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G34" s="11">
+        <v>1</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J34" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K34" s="32"/>
+    </row>
+    <row r="35" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G35" s="10">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="I35" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="J35" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K35" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="K4:K35"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="I6:I9"/>
+    <mergeCell ref="J6:J9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{400D1ED3-44A7-49E9-A961-E022D71E5837}">
   <dimension ref="A6:M30"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
@@ -3216,7 +3841,7 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="21" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -3230,7 +3855,7 @@
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="22" t="s">
         <v>207</v>
       </c>
       <c r="I7" s="7" t="s">
@@ -3246,7 +3871,7 @@
       <c r="M7" s="7"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
+      <c r="A8" s="21"/>
       <c r="B8" s="7" t="s">
         <v>176</v>
       </c>
@@ -3258,7 +3883,7 @@
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
-      <c r="H8" s="23"/>
+      <c r="H8" s="24"/>
       <c r="I8" s="7" t="s">
         <v>187</v>
       </c>
@@ -3272,23 +3897,23 @@
       <c r="M8" s="7"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="20"/>
-      <c r="B9" s="24">
+      <c r="A9" s="21"/>
+      <c r="B9" s="16">
         <v>13</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="D9" s="24">
-        <v>0</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" s="21" t="s">
+      <c r="D9" s="16">
+        <v>0</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="22" t="s">
         <v>19</v>
       </c>
       <c r="I9" s="7" t="s">
@@ -3304,7 +3929,7 @@
       <c r="M9" s="7"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="20"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="7">
         <v>12</v>
       </c>
@@ -3316,7 +3941,7 @@
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
-      <c r="H10" s="22"/>
+      <c r="H10" s="23"/>
       <c r="I10" s="7" t="s">
         <v>189</v>
       </c>
@@ -3330,7 +3955,7 @@
       <c r="M10" s="7"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
+      <c r="A11" s="21"/>
       <c r="B11" s="4">
         <v>11</v>
       </c>
@@ -3343,28 +3968,28 @@
       <c r="E11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="22"/>
-      <c r="I11" s="24">
+      <c r="F11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="23"/>
+      <c r="I11" s="16">
         <v>19</v>
       </c>
-      <c r="J11" s="24" t="s">
+      <c r="J11" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="K11" s="24">
-        <v>0</v>
-      </c>
-      <c r="L11" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="M11" s="24" t="s">
+      <c r="K11" s="16">
+        <v>0</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M11" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="7">
         <v>10</v>
       </c>
@@ -3376,23 +4001,23 @@
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="24">
+      <c r="H12" s="23"/>
+      <c r="I12" s="16">
         <v>18</v>
       </c>
-      <c r="J12" s="24" t="s">
+      <c r="J12" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="K12" s="24">
-        <v>0</v>
-      </c>
-      <c r="L12" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="M12" s="24"/>
+      <c r="K12" s="16">
+        <v>0</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M12" s="16"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
+      <c r="A13" s="21"/>
       <c r="B13" s="4">
         <v>9</v>
       </c>
@@ -3408,7 +4033,7 @@
       <c r="F13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H13" s="22"/>
+      <c r="H13" s="23"/>
       <c r="I13" s="7">
         <v>17</v>
       </c>
@@ -3422,7 +4047,7 @@
       <c r="M13" s="7"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
+      <c r="A14" s="21"/>
       <c r="B14" s="7">
         <v>8</v>
       </c>
@@ -3434,25 +4059,25 @@
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="24">
+      <c r="H14" s="23"/>
+      <c r="I14" s="16">
         <v>16</v>
       </c>
-      <c r="J14" s="24" t="s">
+      <c r="J14" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="K14" s="24">
-        <v>0</v>
-      </c>
-      <c r="L14" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="M14" s="24" t="s">
+      <c r="K14" s="16">
+        <v>0</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M14" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="20"/>
+      <c r="A15" s="21"/>
       <c r="B15" s="4">
         <v>7</v>
       </c>
@@ -3465,10 +4090,10 @@
       <c r="E15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F15" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="22"/>
+      <c r="F15" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="23"/>
       <c r="I15" s="4">
         <v>15</v>
       </c>
@@ -3486,7 +4111,7 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="20"/>
+      <c r="A16" s="21"/>
       <c r="B16" s="7">
         <v>6</v>
       </c>
@@ -3498,7 +4123,7 @@
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
-      <c r="H16" s="22"/>
+      <c r="H16" s="23"/>
       <c r="I16" s="7">
         <v>14</v>
       </c>
@@ -3512,7 +4137,7 @@
       <c r="M16" s="7"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="20"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="4">
         <v>5</v>
       </c>
@@ -3528,7 +4153,7 @@
       <c r="F17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="23"/>
       <c r="I17" s="4">
         <v>13</v>
       </c>
@@ -3546,7 +4171,7 @@
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="20"/>
+      <c r="A18" s="21"/>
       <c r="B18" s="7">
         <v>4</v>
       </c>
@@ -3558,7 +4183,7 @@
       </c>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
-      <c r="H18" s="22"/>
+      <c r="H18" s="23"/>
       <c r="I18" s="4">
         <v>12</v>
       </c>
@@ -3576,7 +4201,7 @@
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="20"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="4">
         <v>3</v>
       </c>
@@ -3589,10 +4214,10 @@
       <c r="E19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F19" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" s="22"/>
+      <c r="F19" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="23"/>
       <c r="I19" s="4">
         <v>11</v>
       </c>
@@ -3605,12 +4230,12 @@
       <c r="L19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="M19" s="24" t="s">
+      <c r="M19" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="20"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="7">
         <v>2</v>
       </c>
@@ -3622,7 +4247,7 @@
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
-      <c r="H20" s="22"/>
+      <c r="H20" s="23"/>
       <c r="I20" s="7">
         <v>10</v>
       </c>
@@ -3636,7 +4261,7 @@
       <c r="M20" s="7"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="20"/>
+      <c r="A21" s="21"/>
       <c r="B21" s="4">
         <v>1</v>
       </c>
@@ -3652,7 +4277,7 @@
       <c r="F21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H21" s="22"/>
+      <c r="H21" s="23"/>
       <c r="I21" s="4">
         <v>9</v>
       </c>
@@ -3670,7 +4295,7 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="20"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="7">
         <v>0</v>
       </c>
@@ -3682,7 +4307,7 @@
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
-      <c r="H22" s="22"/>
+      <c r="H22" s="23"/>
       <c r="I22" s="4">
         <v>8</v>
       </c>
@@ -3700,7 +4325,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H23" s="22"/>
+      <c r="H23" s="23"/>
       <c r="I23" s="4">
         <v>7</v>
       </c>
@@ -3718,7 +4343,7 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H24" s="22"/>
+      <c r="H24" s="23"/>
       <c r="I24" s="4">
         <v>6</v>
       </c>
@@ -3736,7 +4361,7 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H25" s="22"/>
+      <c r="H25" s="23"/>
       <c r="I25" s="4">
         <v>5</v>
       </c>
@@ -3754,7 +4379,7 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H26" s="22"/>
+      <c r="H26" s="23"/>
       <c r="I26" s="4">
         <v>4</v>
       </c>
@@ -3772,7 +4397,7 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H27" s="22"/>
+      <c r="H27" s="23"/>
       <c r="I27" s="4">
         <v>3</v>
       </c>
@@ -3790,7 +4415,7 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H28" s="22"/>
+      <c r="H28" s="23"/>
       <c r="I28" s="4">
         <v>2</v>
       </c>
@@ -3808,7 +4433,7 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H29" s="22"/>
+      <c r="H29" s="23"/>
       <c r="I29" s="4">
         <v>1</v>
       </c>
@@ -3826,7 +4451,7 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H30" s="23"/>
+      <c r="H30" s="24"/>
       <c r="I30" s="4">
         <v>0</v>
       </c>

</xml_diff>